<commit_message>
added cliente_telefone_numero_x/ cliente_telefone_tipo_x descriptions
</commit_message>
<xml_diff>
--- a/Planilhas_importação/Importacao_clientes.xlsx
+++ b/Planilhas_importação/Importacao_clientes.xlsx
@@ -212,8 +212,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Opcional. Informe o órgão emissor do documento de identificação cliente.
-Ex.: SSP</t>
+          <t xml:space="preserve">Informar BR ou UF.</t>
         </r>
       </text>
     </comment>
@@ -267,7 +266,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Obrigatório. Informe o tipo de telefone para contato com o cliente:
+          <t xml:space="preserve">Opicional. Informe o tipo de telefone para contato com o cliente:
 - CELULAR
 - FIXO
 - COMERCIAL
@@ -283,9 +282,40 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Obrigatório. Informar utilizando o padrão a seguir:
+          <t xml:space="preserve">Opicional.  Informar utilizando o padrão a seguir:
 Celular: 5573999341121
 Telefone fixo: 557330130001</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="U1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Opicional. Informe o tipo de telefone para contato com o cliente:
+- CELULAR
+- FIXO
+- COMERCIAL
+-RESIDENCIAL</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="V1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Opicional.  Informar utilizando o padrão a seguir:
+Celular: 5573999341121
+Telefone fixo: 557330130001
+</t>
         </r>
       </text>
     </comment>
@@ -1174,7 +1204,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="33">
+  <cellStyleXfs count="34">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1234,6 +1264,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
@@ -1247,7 +1280,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="32" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="33" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1272,7 +1305,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="19">
+  <cellStyles count="20">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="15" builtinId="3"/>
     <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
@@ -1291,7 +1324,8 @@
     <cellStyle name="Normal" xfId="29"/>
     <cellStyle name="Título de tabela" xfId="30"/>
     <cellStyle name="Índice" xfId="31"/>
-    <cellStyle name="Destaque 3" xfId="32"/>
+    <cellStyle name="caption" xfId="32"/>
+    <cellStyle name="Destaque 3" xfId="33"/>
   </cellStyles>
   <colors>
     <indexedColors>

</xml_diff>